<commit_message>
Update audit log for week 2 and week 3
Week 2 entries covering Use Case Diagram for WriteWise project (actor identification, include/extend relationships, diagram review).
Week 3 entries covering Class Diagram for Assignment 3 (entity classes, composition vs aggregation, repository pattern, diagram review with corrections).
</commit_message>
<xml_diff>
--- a/AI Audit Log_PhamTanHai.xlsx
+++ b/AI Audit Log_PhamTanHai.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -9,77 +9,46 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-100" yWindow="-100" windowWidth="19400" windowHeight="11480" activeTab="1"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="19395" windowHeight="11475" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
-    <sheet name="Assignment 1" sheetId="2" r:id="rId2"/>
-    <sheet name="Assignment 2" sheetId="3" r:id="rId3"/>
-    <sheet name="Assignment 3" sheetId="4" r:id="rId4"/>
+    <sheet name="Week1" sheetId="2" r:id="rId2"/>
+    <sheet name="Week2" sheetId="3" r:id="rId3"/>
+    <sheet name="Week3" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="57">
+  <si>
+    <t>STT</t>
+  </si>
+  <si>
+    <t>Giai đoạn/Thành phần DTC</t>
+  </si>
+  <si>
+    <t>Nội dung Prompt (Câu lệnh)</t>
+  </si>
+  <si>
+    <t>Phản hồi của AI &amp; Quyết định của người học (Reflection)</t>
+  </si>
   <si>
     <t>Ví dụ: Abstraction</t>
   </si>
   <si>
     <t>“Tôi cần quản lý thông tin sinh viên cho app quản lý điểm. Hãy liệt kê các thuộc tính cần thiết."</t>
-  </si>
-  <si>
-    <t>Ví dụ: Process/Algorithm</t>
-  </si>
-  <si>
-    <t>Ví dụ: Pattern Recognition</t>
-  </si>
-  <si>
-    <t>“So sánh các giải thuật CPU scheduling: FCFS, SJF, Round Robin, Priority. Giải thuật nào tốt nhất?”</t>
-  </si>
-  <si>
-    <t>Ví dụ: Pattern Recognition + Literature Review</t>
-  </si>
-  <si>
-    <t>“Tóm tắt 5 bài báo gần đây nhất về anomaly detection trong IoT sensor data.”</t>
-  </si>
-  <si>
-    <t>Giai đoạn/Thành phần DTC</t>
-  </si>
-  <si>
-    <t>Nội dung Prompt (Câu lệnh)</t>
-  </si>
-  <si>
-    <t>Phản hồi của AI &amp; Quyết định của người học (Reflection)</t>
-  </si>
-  <si>
-    <t>STT</t>
   </si>
   <si>
     <t>Phản hồi: AI liệt kê 20 thuộc tính.
 Quyết định: Tôi chỉ chọn 10 thuộc tính liên quan đến chức năng đang được yêu cầu từ ứng dụng (CCCD, địa chỉ...) và lược bỏ 10 thuộc tính học thuật vì phù hợp với yêu cầu của ứng dụng</t>
   </si>
   <si>
+    <t>Ví dụ: Process/Algorithm</t>
+  </si>
+  <si>
     <t>"Viết hàm C sắp xếp mảng sinh viên theo điểm số bằng Selection Sort."</t>
   </si>
   <si>
@@ -87,10 +56,22 @@
 Kiểm chứng: Tôi nhận thấy code AI chưa xử lý trường hợp mảng rỗng (Oversimplification). Tôi đã yêu cầu AI tối ưu lại và tự tay bổ sung điều kiện kiểm tra lỗi.</t>
   </si>
   <si>
+    <t>Ví dụ: Pattern Recognition</t>
+  </si>
+  <si>
+    <t>“So sánh các giải thuật CPU scheduling: FCFS, SJF, Round Robin, Priority. Giải thuật nào tốt nhất?”</t>
+  </si>
+  <si>
     <t>Phản hồi: AI response Round Robin là “tốt nhất” vì cân bằng giữa throughput và fairness.
 Kiểm chứng: AI đưa kết luận sai – không có giải thuật “tốt nhất” tuyệt đối (Hallucination). Mỗi giải thuật phù hợp với tình huống/context khác nhau.</t>
   </si>
   <si>
+    <t>Ví dụ: Pattern Recognition + Literature Review</t>
+  </si>
+  <si>
+    <t>“Tóm tắt 5 bài báo gần đây nhất về anomaly detection trong IoT sensor data.”</t>
+  </si>
+  <si>
     <t>Phản hồi: AI tóm tắt 5 papers với tên tác giả, năm xuất bản và tóm tắt nội dung.
 Kiểm chứng: Tìm trên Google Scholar: 2/5 papers AI nêu là không tồn tại (fabrication). Tôi đã thay bằng 2 papers mà tôi đã tìm kiếm trên research gates và đã kiểm chứng trên google scholar.</t>
   </si>
@@ -130,13 +111,130 @@
   <si>
     <t>Phản hồi: AI đánh giá Microservices là xu hướng "tốt hơn" vì khả năng mở rộng.
 Quyết định: AI đưa kết luận hơi phiến diện (Oversimplification). Thảo luận lớp cho thấy Microservices gây tốn kém chi phí vận hành và phức tạp trong quản lý dữ liệu. Tôi quyết định chọn Monolithic cho dự án nhỏ vì tính đơn giản và tốc độ triển khai nhanh.</t>
+  </si>
+  <si>
+    <t>DECISION-MAKING | DTC: Abstraction – Xác định Actor và phạm vi hệ thống WriteWise</t>
+  </si>
+  <si>
+    <t>"Dự án WriteWise của nhóm tôi là hệ thống luyện kỹ năng viết tiếng Anh. Từ yêu cầu hệ thống, hãy giúp tôi xác định các actor chính cho Use Case Diagram. Hệ thống có các đối tượng: người dùng chưa đăng ký, người dùng đã đăng ký, người dùng trả phí (Premium), quản trị viên và AI Engine chấm bài."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI liệt kê 4 actor: Guest, Registered User, Admin, AI Engine. AI gợi ý Guest chỉ có thể đăng ký tài khoản, Registered User có toàn quyền, Admin quản lý hệ thống.
+Quyết định: AI bỏ sót actor Premium User – đây là một actor riêng biệt với các chức năng đặc thù như Export grading report, View grammar weakness profile, View personal vocabulary book, View error-frequency &amp; topic-coverage chart, Take quiz. Tôi bổ sung Premium User vào diagram và xác định rõ quan hệ kế thừa: Registered User là base actor, Premium User kế thừa từ Registered User (dùng generalization). Quyết định này ảnh hưởng trực tiếp đến cách phân nhóm use case và phân quyền trong hệ thống.</t>
+  </si>
+  <si>
+    <t>VERIFICATION | DTC: Pattern Recognition – Phân loại quan hệ Include, Extend trong Use Case</t>
+  </si>
+  <si>
+    <t>"Trong WriteWise, use case "Write essay" của Registered User có thể kéo theo "Use timed exam mode" (nếu người dùng chọn). Còn "Submit essay for grading" thì luôn kéo theo "Grade essay" (do AI Engine thực hiện). Tôi nên dùng quan hệ Include hay Extend cho từng cặp? Giải thích theo chuẩn UML."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích đúng: &lt;&lt;include&gt;&gt; cho hành vi bắt buộc luôn xảy ra, &lt;&lt;extend&gt;&gt; cho hành vi tùy chọn có điều kiện. AI gợi ý: "Write essay &lt;&lt;extend&gt;&gt; Use timed exam mode" và "Submit essay for grading &lt;&lt;include&gt;&gt; Grade essay".
+Kiểm chứng: Tôi đối chiếu với Ch06 slide 18 – AI trả lời đúng nguyên tắc. Tuy nhiên AI không nêu rõ "Use timed exam mode" phải có extension point cụ thể (ví dụ: [if user activates timed mode]). Quyết định: Tôi giữ đúng cách phân loại của AI nhưng bổ sung thêm điều kiện extension point vào diagram. Đồng thời xác nhận thêm: "Grade essay &lt;&lt;include&gt;&gt; Classify grammar errors", "Grade essay &lt;&lt;include&gt;&gt; Analyze grammar mistakes", "Grade essay &lt;&lt;include&gt;&gt; Suggest vocabulary upgrade" là ba include bắt buộc vì AI Engine luôn thực hiện đủ 3 bước khi chấm bài.</t>
+  </si>
+  <si>
+    <t>PROBLEM-SOLVING | DTC: Decomposition – Phân nhóm Use Case cho WriteWise</t>
+  </si>
+  <si>
+    <t>"Hệ thống WriteWise có nhiều use case cho 5 actor khác nhau (Guest, Registered User, Premium User, Admin, AI Engine). Theo Ch06, tôi nên tổ chức các use case như thế nào trong một diagram duy nhất để đảm bảo dễ đọc và không bị rối? Có nên tách thành nhiều diagram không?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI gợi ý vẽ tất cả vào 1 diagram và nhóm use case theo actor để dễ nhìn. AI cho rằng hệ thống WriteWise không quá phức tạp nên 1 diagram là đủ.
+Quyết định: Tôi đánh giá lại – WriteWise có ~30 use case phân bố trên 5 actor với các nhóm chức năng rõ ràng: nhóm quản lý bài viết, nhóm chấm bài AI, nhóm quản lý ngữ pháp, nhóm tính năng Premium, nhóm quản trị Admin. Sau khi vẽ thử, 1 diagram vẫn đủ rõ ràng vì các actor được bố trí hai bên (Guest/Registered User/Premium User ở trái, Admin ở phải, AI Engine ở phải dưới), các use case được nhóm theo chiều dọc tương ứng với từng actor. Tôi giữ nguyên 1 diagram nhưng tối ưu layout, đặt use case Premium User ở phần dưới riêng biệt để phân biệt với Registered User thông thường. Không cần tách vì scope vừa phải, tách ra sẽ làm mất thấy mối liên hệ giữa các actor.</t>
+  </si>
+  <si>
+    <t>VERIFICATION | DTC: Pattern Recognition – Quan hệ Generalization giữa các Actor</t>
+  </si>
+  <si>
+    <t>"Trong WriteWise, Guest có thể đăng ký tài khoản để trở thành Registered User, và Registered User có thể nâng cấp thành Premium User. Tôi có nên dùng quan hệ Generalization giữa 3 actor này không? Ký hiệu và ý nghĩa UML của Generalization giữa actor là gì theo Ch06?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích Generalization giữa actor thể hiện quan hệ "is-a" – subactor thừa hưởng toàn bộ use case của superactor và có thêm use case riêng. AI gợi ý: Guest ◁ Registered User ◁ Premium User.
+Kiểm chứng: Tôi tra Ch06 slide 13 và 18 – AI đúng về định nghĩa. Nhưng tôi nhận thấy Guest KHÔNG phải là một dạng "is-a" của Registered User; Guest là người chưa xác thực còn Registered User là người đã xác thực – đây là 2 trạng thái, không phải quan hệ kế thừa thực sự. Quyết định: Tôi CHỈ dùng Generalization giữa Registered User ◁ Premium User (vì Premium User IS-A Registered User có thêm đặc quyền), còn Guest là actor độc lập chỉ có 2 use case (Register account, Login/Logout). Cách này phản ánh đúng ngữ nghĩa của hệ thống và tránh lạm dụng Generalization.</t>
+  </si>
+  <si>
+    <t>VERIFICATION | DTC: Evaluation – Gửi Use Case Diagram WriteWise để AI nhận xét</t>
+  </si>
+  <si>
+    <t>[Đính kèm ảnh Use Case Diagram WriteWise]
+"Đây là Use Case Diagram của dự án WriteWise mà tôi đã vẽ. Hãy nhận xét diagram này theo các tiêu chí: (1) Actor và phân quyền có đúng không? (2) Các quan hệ Include/Extend/Generalization có được áp dụng đúng chuẩn UML không? (3) Có use case nào bị thừa, thiếu hoặc đặt sai actor không? (4) Layout và cách tổ chức diagram có rõ ràng không?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI nhận xét tổng thể diagram WriteWise khá đầy đủ và có cấu trúc rõ ràng. AI chỉ ra một số điểm cần cải thiện:
+(1) Actor: Xác định đúng 5 actor (Guest, Registered User, Premium User, Admin, AI Engine). Quan hệ Generalization Registered User ◁ Premium User được vẽ đúng. Tuy nhiên AI gợi ý cần kiểm tra lại xem Guest có thực sự cần 2 use case riêng hay chỉ cần 1.
+(2) Quan hệ: Các &lt;&lt;include&gt;&gt; giữa "Grade essay" và 3 use case con (Classify grammar errors, Analyze grammar mistakes, Suggest vocabulary upgrade) được áp dụng đúng. Tuy nhiên "Generate quiz from errors &amp; vocab" nên được nối bằng &lt;&lt;include&gt;&gt; từ "Grade essay" thay vì đứng độc lập, vì quiz được tạo ra từ kết quả chấm bài.
+(3) AI phát hiện "Change user plans" ở phần Admin có thể cần thêm quan hệ rõ hơn – use case này ảnh hưởng đến Premium User nhưng không có mũi tên liên hệ.
+(4) Layout: AI đánh giá cách sắp xếp 2 cột (trái: user actors, phải: admin và AI) là hợp lý, giúp người đọc phân biệt được nhóm chức năng.
+Quyết định: Tôi chấp nhận góp ý (2) về "Generate quiz" – đây là lỗi thiếu quan hệ. Tôi bổ sung &lt;&lt;include&gt;&gt; từ "Grade essay" → "Generate quiz from errors &amp; vocab". Về điểm (3), tôi giải thích "Change user plans" là chức năng Admin quản lý gói dịch vụ, không cần nối trực tiếp với Premium User vì đây là tác vụ backend. Giữ nguyên layout. Kết quả: diagram được cập nhật 1 thay đổi nhỏ nhưng có giá trị về mặt UML.</t>
+  </si>
+  <si>
+    <t>DECISION-MAKING | DTC: Abstraction – Xác định các lớp chính cho Class Diagram WriteWise</t>
+  </si>
+  <si>
+    <t>"Dự án WriteWise là hệ thống luyện kỹ năng viết tiếng Anh tích hợp AI chấm bài. Theo Ch07 Static Modeling, hãy giúp tôi xác định các entity class chính cần có trong Class Diagram. Hệ thống có các tính năng: viết bài luận, nộp bài để AI chấm, xem lịch sử bài nộp, quản lý ngữ pháp, quản lý từ vựng, thi có hẹn giờ, và tính năng Premium."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI liệt kê các entity class: User, Essay, Submission, GrammarError, Topic, WritingType, GrammarCategory, TheoryNote, VocabBook.
+Quyết định: AI bỏ sót một số class quan trọng phản ánh đúng domain WriteWise: GradingResult (kết quả chấm bài với điểm số và nhận xét tổng thể), Quiz (bài kiểm tra sinh từ lỗi ngữ pháp/từ vựng), QuizResult (kết quả làm quiz), UserPlan (gói dịch vụ Premium của người dùng). Ngoài ra AI gộp Submission và Essay thành 1 nhưng thực ra Essay là bài viết gốc, Submission là hành động nộp bài để chấm (1 Essay có thể nộp lại nhiều lần). Tôi tách ra để phản ánh đúng nghiệp vụ. Quyết định bổ sung 4 class còn thiếu và tách Essay/Submission thành 2 class riêng.</t>
+  </si>
+  <si>
+    <t>VERIFICATION | DTC: Pattern Recognition – Phân biệt Composition và Aggregation trong WriteWise</t>
+  </si>
+  <si>
+    <t>"Trong WriteWise, Submission chứa nhiều GrammarError (lỗi được phát hiện khi chấm bài), còn GrammarCategory có thể chứa nhiều TheoryNote (ghi chú lý thuyết). Quan hệ nào là Composition, quan hệ nào là Aggregation? Giải thích theo tiêu chí vòng đời (lifecycle) và tính độc quyền (exclusivity) theo Ch07."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI trả lời cả hai đều là Composition vì đều là "whole/part".
+Kiểm chứng: AI SAI ở vế GrammarCategory – TheoryNote. Tôi tra Ch07 slide 13-14: Composition = bộ phận sống/chết cùng toàn thể và chỉ thuộc MỘT toàn thể; Aggregation = bộ phận có thể thuộc nhiều toàn thể và sống độc lập. Một TheoryNote (ví dụ: giải thích về Present Perfect) có thể được gắn vào nhiều GrammarCategory khác nhau bởi Admin, và xóa một GrammarCategory không nên xóa TheoryNote. Đây rõ ràng là Aggregation. Ngược lại, GrammarError chỉ thuộc về 1 Submission cụ thể và mất đi khi Submission bị xóa – đây là Composition đúng nghĩa.
+Quyết định: Submission ◆── GrammarError = COMPOSITION; GrammarCategory ◇── TheoryNote = AGGREGATION. Bổ sung kiểm chứng bằng logic nghiệp vụ: nếu bỏ 1 Submission, GrammarError liên quan cũng không còn ý nghĩa; nhưng TheoryNote vẫn còn giá trị dù GrammarCategory bị vô hiệu hóa.</t>
+  </si>
+  <si>
+    <t>PROBLEM-SOLVING | DTC: Abstraction – Thiết kế quan hệ Inheritance cho User trong WriteWise</t>
+  </si>
+  <si>
+    <t>"Trong WriteWise, có 2 loại người dùng: Registered User (người dùng thường) và Premium User (trả phí). Premium User có thêm các tính năng: Export grading report, View grammar weakness profile, View personal vocabulary book, View error-frequency chart, Take quiz. Tôi nên dùng Generalization (superclass User – subclass RegisteredUser, PremiumUser) hay chỉ dùng 1 class User với field IsPremium? Theo Ch07, cách nào đúng hơn về mặt UML?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI khuyên dùng Generalization hierarchy: superclass User kế thừa xuống RegisteredUser và PremiumUser. AI cho rằng đây là chuẩn OOP và Ch07.
+Quyết định: Về lý thuyết Ch07 slide 15-16, AI đúng – PremiumUser là một "is-a" User với thêm method riêng. Tuy nhiên trong thực tế WriteWise, sự khác biệt giữa 2 loại user chủ yếu là về QUYỀN TRUY CẬP tính năng, không phải khác biệt về cấu trúc dữ liệu. Cả hai đều có email, password, profile giống nhau. Tôi quyết định: (1) Ở analysis class diagram → vẽ Generalization hierarchy User ◁ RegisteredUser ◁ PremiumUser để đúng lý thuyết Ch07 và phản ánh quan hệ "is-a" có ý nghĩa ngữ nghĩa. (2) Ở design level → có thể dùng 1 class User + field UserPlan để dễ implement. Ghi chú trade-off rõ trong báo cáo.</t>
+  </si>
+  <si>
+    <t>VERIFICATION | DTC: Pattern Recognition – Áp dụng Repository Pattern cho WriteWise Class Diagram</t>
+  </si>
+  <si>
+    <t>"Đề bài Assignment 3 yêu cầu thiết kế Class Diagram theo Repository Pattern để tách business logic khỏi data access logic. Theo Ch07 và yêu cầu đề, tôi cần có: IRepository interface, SubmissionRepository, GradingService. Hãy giải thích mối quan hệ Dependency giữa GradingService và SubmissionRepository theo UML. Ký hiệu dependency trong class diagram là gì?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích đúng: Dependency (mũi tên đứt nét ──►) dùng khi một class "sử dụng" class khác nhưng không sở hữu nó. GradingService phụ thuộc vào SubmissionRepository vì cần gọi method để truy xuất dữ liệu Submission khi chấm bài. AI cũng đề cập: Repository classes implement interface IRepository&lt;T&gt; dùng ký hiệu "realize" (mũi tên đứt nét tam giác rỗng).
+Kiểm chứng: Khớp với yêu cầu đề bài và nguyên tắc UML. Tuy nhiên AI không làm rõ sự khác biệt giữa Dependency và Association – cả hai đều có mũi tên nhưng Association là quan hệ cấu trúc lâu dài (có thuộc tính), còn Dependency là quan hệ sử dụng tạm thời (tham số method, biến cục bộ).
+Quyết định: Tôi áp dụng Dependency cho GradingService → SubmissionRepository và GradingService → GradingResultRepository. Sử dụng Realization (──▷) cho SubmissionRepository implements IRepository&lt;Submission&gt;. Bổ sung vào diagram chú thích rõ để phân biệt Association và Dependency tránh nhầm lẫn khi trình bày.</t>
+  </si>
+  <si>
+    <t>VERIFICATION | DTC: Evaluation – Gửi Class Diagram Assignment 3 để AI nhận xét và phát hiện lỗi</t>
+  </si>
+  <si>
+    <t>[Đính kèm ảnh Class Diagram Assignment 3 – Car Rental System]
+"Đây là Class Diagram thiết kế cho bài Assignment 3 (Car Rental System theo Repository Pattern). Hãy nhận xét và chỉ ra các lỗi sai (nếu có) về: (1) Quan hệ Inheritance/Realization có đúng không? (2) Multiplicity của các quan hệ Association/Aggregation/Composition có hợp lý không? (3) Dependency giữa Service layer và Repository layer có được thể hiện đúng không? (4) Có class hoặc interface nào bị thiếu theo yêu cầu đề không?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI nhận xét Class Diagram theo từng tiêu chí:
+(1) Inheritance: Customer và Staff kế thừa từ User – đúng yêu cầu đề. Tuy nhiên AI phát hiện lỗi: cần kiểm tra lại ký hiệu – Inheritance dùng mũi tên tam giác đặc (──▶) không đứt nét, còn Realization dùng mũi tên tam giác rỗng đứt nét (⋯▷). Nếu diagram dùng nhầm ký hiệu sẽ bị sai về mặt UML.
+(2) Multiplicity: Quan hệ Customer – Booking (1 đến nhiều) là đúng. Booking – Car (nhiều Booking – 1 Car) cần kiểm tra có ghi multiplicity ở cả 2 đầu không – AI thấy một số đầu bị thiếu nhãn.
+(3) Dependency: GradingService → Repository được thể hiện bằng mũi tên đứt nét – đúng. Tuy nhiên AI gợi ý tên mũi tên nên có stereotype &lt;&lt;use&gt;&gt; hoặc &lt;&lt;call&gt;&gt; để rõ ràng hơn.
+(4) AI phát hiện thiếu: Interface IRepository&lt;T&gt; cần được vẽ với stereotype &lt;&lt;interface&gt;&gt; rõ ràng; PaymentService chưa có dependency rõ ràng đến PaymentRepository.
+Quyết định: Tôi xem xét và sửa các lỗi sau:
+• Kiểm tra lại toàn bộ ký hiệu Inheritance vs Realization – đây là lỗi dễ gây mất điểm nhất.
+• Bổ sung multiplicity còn thiếu ở các đầu quan hệ Booking–Car.
+• Thêm stereotype &lt;&lt;interface&gt;&gt; vào IRepository&lt;T&gt;.
+• Bổ sung dependency PaymentService → PaymentRepository.
+Không áp dụng gợi ý stereotype &lt;&lt;use&gt;&gt; vì theo Ch07 không yêu cầu label cho dependency thông thường.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -153,6 +251,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -162,7 +269,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -185,11 +292,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -208,6 +330,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -544,80 +672,80 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="20.9140625" customWidth="1"/>
-    <col min="2" max="2" width="26.83203125" customWidth="1"/>
+    <col min="1" max="1" width="20.875" customWidth="1"/>
+    <col min="2" max="2" width="26.875" customWidth="1"/>
     <col min="3" max="3" width="24.25" customWidth="1"/>
     <col min="4" max="4" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" ht="15">
       <c r="A1" s="5" t="s">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" spans="1:5" ht="70">
+    <row r="2" spans="1:5" ht="69.95" customHeight="1">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="56">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="56.1" customHeight="1">
       <c r="A3" s="2">
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="70">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="69.95" customHeight="1">
       <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="84">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="84" customHeight="1">
       <c r="A5" s="2">
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>15</v>
@@ -631,29 +759,29 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="20.9140625" customWidth="1"/>
-    <col min="2" max="2" width="26.83203125" customWidth="1"/>
+    <col min="1" max="1" width="20.875" customWidth="1"/>
+    <col min="2" max="2" width="26.875" customWidth="1"/>
     <col min="3" max="3" width="24.25" customWidth="1"/>
     <col min="4" max="4" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" ht="15">
       <c r="A1" s="5" t="s">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="140">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="140.1" customHeight="1">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -667,12 +795,12 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="126">
+    <row r="3" spans="1:4" ht="126" customHeight="1">
       <c r="A3" s="2">
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>19</v>
@@ -681,7 +809,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="126">
+    <row r="4" spans="1:4" ht="126" customHeight="1">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -695,7 +823,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="140">
+    <row r="5" spans="1:4" ht="140.1" customHeight="1">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -716,18 +844,200 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14"/>
-  <sheetData/>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="40" customWidth="1"/>
+    <col min="4" max="4" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="15">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="159.94999999999999" customHeight="1">
+      <c r="A2" s="8">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="174.95" customHeight="1">
+      <c r="A3" s="8">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="174.95" customHeight="1">
+      <c r="A4" s="8">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="174.95" customHeight="1">
+      <c r="A5" s="8">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="200.1" customHeight="1">
+      <c r="A6" s="8">
+        <v>5</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14"/>
-  <sheetData/>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="40" customWidth="1"/>
+    <col min="4" max="4" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="15">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="165" customHeight="1">
+      <c r="A2" s="8">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="200.1" customHeight="1">
+      <c r="A3" s="8">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="189.95" customHeight="1">
+      <c r="A4" s="8">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="195" customHeight="1">
+      <c r="A5" s="8">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="230.1" customHeight="1">
+      <c r="A6" s="8">
+        <v>5</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Audit Log Week 4
Sequence Diagram for WriteWise
</commit_message>
<xml_diff>
--- a/AI Audit Log_PhamTanHai.xlsx
+++ b/AI Audit Log_PhamTanHai.xlsx
@@ -9,20 +9,21 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="19395" windowHeight="11475" activeTab="3"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19400" windowHeight="11480" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
     <sheet name="Week1" sheetId="2" r:id="rId2"/>
     <sheet name="Week2" sheetId="3" r:id="rId3"/>
     <sheet name="Week3" sheetId="4" r:id="rId4"/>
+    <sheet name="Week4" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="72">
   <si>
     <t>STT</t>
   </si>
@@ -228,6 +229,61 @@
 • Thêm stereotype &lt;&lt;interface&gt;&gt; vào IRepository&lt;T&gt;.
 • Bổ sung dependency PaymentService → PaymentRepository.
 Không áp dụng gợi ý stereotype &lt;&lt;use&gt;&gt; vì theo Ch07 không yêu cầu label cho dependency thông thường.</t>
+  </si>
+  <si>
+    <t>DECISION-MAKING | DTC: Abstraction – Xác định luồng tương tác chính trong Sequence Diagram “Submit Essay for Grading”</t>
+  </si>
+  <si>
+    <t>“Dự án WriteWise có use case “Submit essay for grading” là luồng quan trọng nhất. Hãy giúp tôi xác định các đối tượng tham gia (lifeline) và thứ tự message cần vẽ trong Sequence Diagram cho luồng này. Hệ thống có: User (trình duyệt), EssayController, GradingService, AI Engine, Database. Hành động: user submit bài viết → hệ thống lưu bài → gọi AI chấm → lưu kết quả → trả về thông báo.”</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI xác định 5 lifeline: User, EssayController, GradingService, AIEngine, Database. Luồng message: User → EssayController: submitEssay(content) → EssayController → Database: saveEssay() → EssayController → GradingService: gradeEssay(essayId) → GradingService → AIEngine: analyze(essayText) → AIEngine → GradingService: return GradingResult → GradingService → Database: saveGradingResult() → EssayController → User: return gradingReport.
+Quyết định: AI đưa ra luồng cơ bản nhưng bỏ sót 3 điểm quan trọng trong nghiệp vụ WriteWise: (1) Không có bước kiểm tra giới hạn submission của Registered User (mỗi bài chỉ được nộp tối đa 3 lần). (2) Không tách biệt luồng phản hồi cho Premium User (được xem báo cáo chi tiết ngay) và Registered User (chỉ xem điểm tổng). (3) Thiếu bước GradingService gọi sub-routine “GenerateQuiz” sau khi chấm xong. Tôi bổ sung 3 điểm này vào diagram: thêm opt fragment kiểm tra submission limit, thêm alt fragment phân biệt phản hồi Premium vs Regular, và bổ sung message GradingService → QuizService: generateQuiz(errors, vocab).</t>
+  </si>
+  <si>
+    <t>VERIFICATION | DTC: Pattern Recognition – Phân biệt Synchronous và Asynchronous Message trong Sequence Diagram WriteWise</t>
+  </si>
+  <si>
+    <t>“Trong Sequence Diagram WriteWise, khi EssayController gọi GradingService.gradeEssay(), quá trình AI chấm bài có thể mất vài giây. Tôi nên dùng Synchronous message (mũi tên liền nét ►) hay Asynchronous message (mũi tên hở &gt;) cho lời gọi này? Theo Ch08, khác biệt kỹ thuật và khi nào nên dùng mỗi loại?”</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích: Synchronous message = người gọi chờ cho đến khi nhận được phản hồi mới tiếp tục (blocking call); Asynchronous message = người gọi gửi rồi tiếp tục luồng khác mà không chờ (non-blocking). AI gợi ý dùng Asynchronous cho grading vì “AI chấm bài lâu”.
+Kiểm chứng: Tôi tra Ch08 slide 10–12 và đánh giá lại theo nghiệp vụ WriteWise. Nếu dùng Async, EssayController phải có cơ chế polling hoặc callback – làm phức tạp hóa diagram và chưa cần thiết ở mức analysis. Theo yêu cầu đề bài chỉ vẽ ở mức analysis-level Sequence Diagram, Synchronous là phù hợp hơn vì nó mô tả rõ luồng xử lý tuần tự dễ hiểu. Asynchronous chỉ cần ở design/implementation level khi xây dựng thực tế. Quyết định: Dùng Synchronous message cho toàn bộ luồng trong Sequence Diagram mức analysis. Ghi chú trong sưu tầm: “ở level implementation có thể chuyển sang Async Job Queue cho GradingService” để thể hiện sự hiểu biết trade-off.</t>
+  </si>
+  <si>
+    <t>PROBLEM-SOLVING | DTC: Decomposition – Thiết kế Sequence Diagram cho luồng “Take Quiz” của Premium User</t>
+  </si>
+  <si>
+    <t>“WriteWise có tính năng “Take quiz” dành cho Premium User: hệ thống tự động tạo quiz từ các lỗi ngữ pháp và từ vựng mà AI phát hiện khi chấm bài. Hãy giúp tôi phân rã luồng này thành các bước trong Sequence Diagram: từ lúc user click “Start Quiz” đến khi xem kết quả. Các đối tượng có: PremiumUser, QuizController, QuizService, QuizRepository, Database.”</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đưa ra luồng 6 bước: PremiumUser → QuizController: startQuiz(submissionId) → QuizController → QuizService: getQuizBySubmission(submissionId) → QuizService → QuizRepository: findBySubmissionId() → QuizRepository → DB: query() → QuizController → PremiumUser: displayQuizUI(questions) → PremiumUser → QuizController: submitAnswers(answers) → QuizController → QuizService: evaluateAnswers() → QuizController → PremiumUser: showResult(score, feedback).
+Quyết định: AI có luồng tốt nhưng chưa xử lý 2 trường hợp: (1) Quiz chưa được tạo sẵn (nếu submission vừa nộp chưa chấm xong) – cần opt fragment báo “Quiz not available yet”. (2) Không có bước kiểm tra quyền Premium User trước khi cho phép truy cập – nếu Registered User cố gọi endpoint này, hệ thống phải từ chối. Tôi bổ sung: (1) alt fragment ở đầu luồng: [isPremium = true] tiếp tục luồng bình thường / [else] QuizController → User: return 403 Forbidden. (2) opt fragment trước displayQuizUI: [quiz not generated] → gọi QuizService.generateQuiz(errors). Đây là 2 điểm bảo vệ tính toàn vẹn luồng và phản ánh đúng nghiệp vụ Premium feature của WriteWise.</t>
+  </si>
+  <si>
+    <t>VERIFICATION | DTC: Pattern Recognition – Sử dụng Combined Fragment (alt, opt, loop) đúng chuẩn UML trong Sequence Diagram</t>
+  </si>
+  <si>
+    <t>“Trong Sequence Diagram của WriteWise, tôi cần biểu diễn: (1) Nếu submission quá giới hạn 3 lần, hệ thống từ chối (dùng alt). (2) Nếu đó là Premium User, truyền thêm thông tin báo cáo chi tiết (dùng opt). (3) GradingService lặp qua từng câu trong bài để phát hiện lỗi (dùng loop). Theo Ch08, ý nghĩa và cú pháp chính xác của từng fragment là gì?”</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích đúng 3 loại: alt = các nhánh điều kiện loại trừ nhau (if-else); opt = khối chỉ thực hiện khi điều kiện đúng (if-only); loop = lặp lại theo điều kiện hoặc số lần. Nhưng AI không đề cập 2 điểm quan trọng: (a) Cú pháp của guard label (có thể viết “[submissionCount ≥ 3]” trên thanh fragment), và (b) Loop được gọi với tham số “loop(1, n)” thể hiện tối thiểu và tối đa số lần lặp.
+Kiểm chứng: Tôi tra Ch08 slide 19–22. Xác nhận: alt dùng ký hiệu thanh nằm ngang chia nhánh, mỗi nhánh có guard condition trong ngoặc vuông. opt là dạng đặc biệt của alt chỉ có 1 nhánh. loop có thể viết “loop(minCount, maxCount)” hoặc chỉ “loop” kèm guard. Quyết định: Tôi áp dụng đúng: alt [submissionCount &lt; 3] / [else return “Limit exceeded”]; opt [isPremium] gọi thêm getDetailedReport(); loop(1, essayLength) GradingService phân tích từng câu. Bổ sung guard condition rõ ràng cho từng fragment, tránh viết guard kiểu “some condition” mơ hồ.</t>
+  </si>
+  <si>
+    <t>VERIFICATION | DTC: Evaluation – Gửi Sequence Diagram WriteWise để AI nhận xét toàn diện</t>
+  </si>
+  <si>
+    <t>[Dính kèm ảnh Sequence Diagram luồng “Submit Essay for Grading” của WriteWise]
+“Đây là Sequence Diagram tôi đã vẽ cho luồng nộp bài và chấm bài của hệ thống WriteWise. Hãy nhận xét theo các tiêu chí: (1) Các lifeline có xác định đúng và đủ không? (2) Thứ tự message có hợp lý theo luồng nghiệp vụ không? (3) Các Combined Fragment (alt, opt, loop) có được áp dụng đúng chuẩn UML không? (4) Có message nào bị thừa, thiếu hoặc có tên không rõ ràng không?”</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI nhận xét Sequence Diagram WriteWise theo từng tiêu chí:
+(1) Lifeline: Xác định đúng 5 đối tượng (User, EssayController, GradingService, AIEngine, Database). AI ghi nhận việc tách GradingService và AIEngine thành 2 lifeline riêng là hợp lý và phản ánh đúng kiến trúc hệ thống. Tuy nhiên AI gợi ý nên thêm QuizService như một lifeline riêng thay vì để trong GradingService để đúng Single Responsibility.
+(2) Thứ tự message: Luồng tuần tự logic (submit → save → grade → generate quiz → return) được đánh giá là hợp lý. AI chỉ ra: Database.saveEssay() và Database.saveGradingResult() nên được đặt tên nhất quán (nên viết rõ là Database: essays.save() và Database: gradingResults.save()).
+(3) Combined Fragment: AI xác nhận alt và opt fragment được áp dụng đúng. Tuy nhiên loop fragment thiếu tham số: viết “loop” đơn lẻ không có guard condition cụ thể (không biết lặp mấy lần hoặc điều kiện dừng là gì).
+(4) Tên message: “return gradingReport” nên đổi thành “displayGradingPage(result)” cho rõ hơn.
+Quyết định: Tôi chấp nhận và sửa 3 điểm: (a) Thêm QuizService làm lifeline riêng. (b) Đổi tên Database message theo convention “table.save()”. (c) Bổ sung guard condition cho loop: “loop [for each sentence in essay]”. Không đổi tên “gradingReport” vì trong nghiệp vụ WriteWise, “report” là thuật ngữ đã được thống nhất trong nhóm. Kết quả: Diagram được cập nhật 3 cải tiến có giá trị về mặt UML và nghiệp vụ.</t>
   </si>
 </sst>
 </file>
@@ -311,7 +367,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -336,6 +392,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -672,15 +731,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="20.875" customWidth="1"/>
-    <col min="2" max="2" width="26.875" customWidth="1"/>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="26.83203125" customWidth="1"/>
     <col min="3" max="3" width="24.25" customWidth="1"/>
     <col min="4" max="4" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15">
+    <row r="1" spans="1:5" ht="15" customHeight="1">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -695,7 +754,7 @@
       </c>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" spans="1:5" ht="69.95" customHeight="1">
+    <row r="2" spans="1:5" ht="70" customHeight="1">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -709,7 +768,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="56.1" customHeight="1">
+    <row r="3" spans="1:5" ht="56.15" customHeight="1">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -723,7 +782,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="69.95" customHeight="1">
+    <row r="4" spans="1:5" ht="70" customHeight="1">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -759,15 +818,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="20.875" customWidth="1"/>
-    <col min="2" max="2" width="26.875" customWidth="1"/>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="26.83203125" customWidth="1"/>
     <col min="3" max="3" width="24.25" customWidth="1"/>
     <col min="4" max="4" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15">
+    <row r="1" spans="1:4" ht="15" customHeight="1">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -781,7 +840,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="140.1" customHeight="1">
+    <row r="2" spans="1:4" ht="140.15" customHeight="1">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -823,7 +882,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="140.1" customHeight="1">
+    <row r="5" spans="1:4" ht="140.15" customHeight="1">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -845,7 +904,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -853,7 +912,7 @@
     <col min="4" max="4" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15">
+    <row r="1" spans="1:4" ht="15" customHeight="1">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -867,7 +926,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="159.94999999999999" customHeight="1">
+    <row r="2" spans="1:4" ht="160" customHeight="1">
       <c r="A2" s="8">
         <v>1</v>
       </c>
@@ -881,7 +940,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="174.95" customHeight="1">
+    <row r="3" spans="1:4" ht="175" customHeight="1">
       <c r="A3" s="8">
         <v>2</v>
       </c>
@@ -895,7 +954,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="174.95" customHeight="1">
+    <row r="4" spans="1:4" ht="175" customHeight="1">
       <c r="A4" s="8">
         <v>3</v>
       </c>
@@ -909,7 +968,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="174.95" customHeight="1">
+    <row r="5" spans="1:4" ht="175" customHeight="1">
       <c r="A5" s="8">
         <v>4</v>
       </c>
@@ -923,7 +982,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="200.1" customHeight="1">
+    <row r="6" spans="1:4" ht="200.15" customHeight="1">
       <c r="A6" s="8">
         <v>5</v>
       </c>
@@ -945,7 +1004,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -953,7 +1012,7 @@
     <col min="4" max="4" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15">
+    <row r="1" spans="1:4" ht="15" customHeight="1">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -981,7 +1040,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="200.1" customHeight="1">
+    <row r="3" spans="1:4" ht="200.15" customHeight="1">
       <c r="A3" s="8">
         <v>2</v>
       </c>
@@ -995,7 +1054,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="189.95" customHeight="1">
+    <row r="4" spans="1:4" ht="190" customHeight="1">
       <c r="A4" s="8">
         <v>3</v>
       </c>
@@ -1023,7 +1082,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="230.1" customHeight="1">
+    <row r="6" spans="1:4" ht="230.15" customHeight="1">
       <c r="A6" s="8">
         <v>5</v>
       </c>
@@ -1035,6 +1094,106 @@
       </c>
       <c r="D6" s="8" t="s">
         <v>56</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultRowHeight="14"/>
+  <cols>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="40" customWidth="1"/>
+    <col min="4" max="4" width="75.08203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="15" customHeight="1">
+      <c r="A1" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="203.5" customHeight="1">
+      <c r="A2" s="8">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="200.15" customHeight="1">
+      <c r="A3" s="8">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="190" customHeight="1">
+      <c r="A4" s="8">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="195" customHeight="1">
+      <c r="A5" s="8">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="230.15" customHeight="1">
+      <c r="A6" s="8">
+        <v>5</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update audit log week 7
SOA component diagram
</commit_message>
<xml_diff>
--- a/AI Audit Log_PhamTanHai.xlsx
+++ b/AI Audit Log_PhamTanHai.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="19395" windowHeight="11475" activeTab="6"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="19395" windowHeight="11475" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
@@ -19,13 +19,14 @@
     <sheet name="Week4" sheetId="5" r:id="rId5"/>
     <sheet name="Week5" sheetId="6" r:id="rId6"/>
     <sheet name="Week6" sheetId="7" r:id="rId7"/>
+    <sheet name="Week7" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="126">
   <si>
     <t>STT</t>
   </si>
@@ -394,6 +395,60 @@
   </si>
   <si>
     <t>AI RESPONSE (Summary): AI khuyên để logic trong Controller cho đơn giản vì dự án sinh viên không cần tách tầng quá kỹ. HUMAN DELTA &amp; REFLECTION: • Critical Thinking [Oversimplification]: Đây là lời khuyên nguy hiểm. Dù là dự án môn học, nhóm đã chọn kiến trúc phân tầng và Repository Pattern; đặt business logic trong Controller sẽ làm sai chính thiết kế đã nộp. Controller dày cũng khó test, khó reuse và khó thay đổi khi thêm Moderator workflow. • Contextualization: Forum + Dictionary + Vocabulary là module có nhiều rule: kiểm tra quyền đăng, validate content, report trùng, trạng thái Post, moderator review. Những rule này phải nằm ở Service để tái sử dụng cho nhiều endpoint. • Creative Synthesis: Tôi trình bày hướng đúng: Controller mỏng nhận request và gọi service; Service xử lý rule Create Post/Report Content; Repository làm data access; DTO tách request/response khỏi entity. Nếu code hiện tại có logic dày ở Controller, tôi ghi nhận là điểm cần refactor thay vì coi là chuẩn. • Decision Ownership: Quyết định bảo vệ layered architecture trong phần giải thích Week 6. Lý do: nhất quán với Package Diagram tuần 5 và thể hiện tư duy thiết kế, không chỉ chạy được chức năng. EVIDENCE: Package Diagram Controllers → Services → Repositories; snippet PostController/CommentService.</t>
+  </si>
+  <si>
+    <t>DECISION-MAKING | DTC: Pattern Recognition – Nhận diện Design Pattern đã dùng trong code IELTSPhobic</t>
+  </si>
+  <si>
+    <t>"Tuần này tôi phụ trách vẽ Component Diagram cho phương án SOA của IELTSPhobic. Hãy giúp tôi xác định các component chính và luồng HTTP Request/Response giữa Learner Site, Admin Site, Mobile App tương lai và IPS Core Service."</t>
+  </si>
+  <si>
+    <t>AI RESPONSE (Summary): AI đề xuất các component gồm Learner Site, Admin Site, Database và một API Server duy nhất, gần giống kiến trúc hiện tại. HUMAN DELTA &amp; REFLECTION: • Critical Thinking [Context Misunderstanding]: Gợi ý này chưa thể hiện điểm mới của SOA. Tuần 7 yêu cầu phương án SOA để giải quyết vấn đề reusability khi sau này thêm Mobile App, nên diagram phải làm rõ IPS Core Service là service dùng chung cho nhiều client. • Contextualization: Phần tôi phụ trách là Component Diagram SOA, không phải Deployment Diagram. Vì vậy trọng tâm là component và message request/response, không phải server vật lý. • Creative Synthesis: Tôi xác định các component chính: Learner Site, Admin Site, Mobile App (future client), IPS Core Service, Database, External Services nếu cần. Ba client đều gọi IPS Core Service qua HTTP/REST API; IPS Core Service xử lý business logic Forum, Dictionary, Vocabulary và truy cập database. • Decision Ownership: Quyết định vẽ IPS Core Service ở trung tâm, các client ở ngoài gọi vào bằng REST API. Lý do: thể hiện rõ mục tiêu SOA là tái sử dụng core service cho nhiều client, đặc biệt Mobile App tương lai. EVIDENCE: Phân công tuần 7 yêu cầu Component Diagram SOA với HTTP Request/Response giữa client và IPS Core Service.</t>
+  </si>
+  <si>
+    <t>VERIFICATION | DTC: Pattern Recognition – Singleton Pattern: định nghĩa và áp dụng đúng</t>
+  </si>
+  <si>
+    <t>"Trong SOA-based solution của IELTSPhobic, IPS Core Service nên được hiểu là một service dùng chung hay là nhiều service nhỏ như microservice? Khi vẽ Component Diagram tuần 7, tôi nên thể hiện ranh giới này thế nào cho đúng?"</t>
+  </si>
+  <si>
+    <t>AI RESPONSE (Summary): AI nói IPS Core Service nên tách thành nhiều service nhỏ như AuthService, ForumService, DictionaryService, PaymentService để đúng tinh thần service-oriented. HUMAN DELTA &amp; REFLECTION: • Critical Thinking [Oversimplification]: Đây là nhầm SOA với Microservice. Tuần 7 là Alternative Architecture: SOA, còn tuần 8 mới là Microservice + Service Discovery. Nếu tách quá nhỏ ngay tuần 7 thì diagram sẽ trùng với tuần 8 và làm mất ranh giới kiến trúc. • Contextualization: SOA trong báo cáo của nhóm hướng đến việc tách core business capability thành một service dùng chung, không nhất thiết chia thành nhiều deployable service độc lập. • Creative Synthesis: Tôi giữ IPS Core Service là một component lớn, bên trong có các logical modules như Forum, Dictionary, Vocabulary, Auth, Exam. Các module này chỉ ghi chú bên trong service hoặc mô tả bằng note, không vẽ thành microservice riêng. • Decision Ownership: Quyết định không tách IPS Core Service thành nhiều microservice ở Week 7. Lý do: giữ đúng phạm vi SOA và để Week 8 xử lý Service Register, API Gateway, nhiều service độc lập. CORRECTIVE ACTION: Vẽ một IPS Core Service dùng chung, không vẽ Service Discovery ở tuần 7. EVIDENCE: Plan tuần 7 SOA; plan tuần 8 Microservice + Service Discovery.</t>
+  </si>
+  <si>
+    <t>PROBLEM-SOLVING | DTC: Pattern Recognition – Strategy Pattern: nhận diện và vẽ class diagram</t>
+  </si>
+  <si>
+    <t>"Hãy đề xuất cách đánh số message trong Component Diagram SOA cho luồng Forum + Dictionary: client gửi request tạo post, tra từ điển, lưu từ vựng; IPS Core Service xử lý và trả response. Nên đánh số theo request/response như thế nào?"</t>
+  </si>
+  <si>
+    <t>AI RESPONSE (Summary): AI đề xuất đánh số message chỉ một chiều: 1. Client sends request, 2. IPS Core Service returns data. HUMAN DELTA &amp; REFLECTION: • Critical Thinking: Cách đánh số này quá sơ sài, chưa giúp người đọc trace từng use case. Vì yêu cầu của tôi là luồng HTTP Request/Response, mỗi chức năng cần có cặp request và response rõ ràng. • Contextualization: Module của tôi gồm Forum + Dictionary + Vocabulary, nên message không chỉ có một request chung mà gồm nhiều endpoint khác nhau: create post, report content, search dictionary, save word. • Creative Synthesis: Tôi đánh số theo cặp: 1. Learner Site -&gt; IPS Core Service: POST /api/forum/posts; 2. IPS Core Service -&gt; Database: Insert Post; 3. IPS Core Service -&gt; Learner Site: 201 Created; 4. Learner Site -&gt; IPS Core Service: GET /api/dictionary?word=...; 5. IPS Core Service -&gt; Database/Dictionary provider: Lookup word; 6. IPS Core Service -&gt; Learner Site: 200 WordDetail; 7. Learner Site -&gt; IPS Core Service: POST /api/vocabulary/saved-words; 8. IPS Core Service -&gt; Learner Site: 200 Saved. • Decision Ownership: Quyết định đánh số message theo từng cặp request/response và có HTTP method/status code. Lý do: diagram rõ luồng hơn và đúng yêu cầu đánh số message. EVIDENCE: Component Diagram SOA Forum + Dictionary flow.</t>
+  </si>
+  <si>
+    <t>VERIFICATION | DTC: Abstraction – Observer Pattern vs Event-driven: phân biệt đúng</t>
+  </si>
+  <si>
+    <t>"AI gợi ý dùng mũi tên dependency tĩnh giữa component là đủ, không cần thể hiện message HTTP request/response. Với yêu cầu của tôi là 'luồng HTTP Request/Response, đánh số message', cách đó có đủ không?"</t>
+  </si>
+  <si>
+    <t>AI RESPONSE (Summary): AI nói Component Diagram chỉ cần dependency arrows giữa components, không cần message numbering vì message thuộc Sequence Diagram. HUMAN DELTA &amp; REFLECTION: • Critical Thinking [Partial Truth]: AI đúng ở mức UML cơ bản: Component Diagram thường thể hiện dependency/interface. Nhưng yêu cầu cụ thể của phần tôi là vẽ Component Diagram SOA thể hiện luồng HTTP Request/Response và đánh số message, nên chỉ có dependency arrows là chưa đủ. • Contextualization: Báo cáo nhóm cần giải thích cách client giao tiếp với IPS Core Service trong kiến trúc SOA. Nếu chỉ vẽ mũi tên phụ thuộc không tên, người đọc không thấy API nào được gọi và SOA giải quyết reuse như thế nào. • Creative Synthesis: Tôi kết hợp hai cách: dùng component boxes và interface/REST API ports theo tinh thần Component Diagram, nhưng label trên connector bằng message đã đánh số: 1 POST /api/forum/posts, 2 201 Created, 3 GET /api/dictionary, 4 200 OK. Như vậy diagram vừa đúng component view vừa đáp ứng yêu cầu luồng message. • Decision Ownership: Quyết định dùng labeled connectors có số thứ tự, không chỉ dependency arrows trống. Lý do: phù hợp requirement của tuần 7 và giúp phân biệt SOA diagram với package diagram tuần 5. EVIDENCE: Yêu cầu 'HTTP Request/Response, đánh số message' trong phân công Phạm Tấn Hải.</t>
+  </si>
+  <si>
+    <t>PROBLEM-SOLVING | DTC: Pattern Recognition – Facade Pattern: đơn giản hóa giao diện phức tạp</t>
+  </si>
+  <si>
+    <t>"Khi chuyển từ kiến trúc hiện tại Multiple Client/Single Server sang SOA, các thay đổi implementation nào liên quan đến client và API cần được phản ánh trong Component Diagram? Ví dụ JWT, Swagger/OpenAPI, CORS, API versioning."</t>
+  </si>
+  <si>
+    <t>AI RESPONSE (Summary): AI chỉ nói chuyển sang SOA nghĩa là đổi database thành shared database và giữ cookie authentication như cũ. HUMAN DELTA &amp; REFLECTION: • Critical Thinking [Oversimplification]: SOA không chỉ là đổi database. Khi nhiều client cùng gọi IPS Core Service, các vấn đề API contract, authentication và cross-origin trở nên quan trọng. Cookie auth phù hợp web monolith hơn, nhưng mobile app tương lai cần token-based auth. • Contextualization: Phần implementation changes của tuần 7 nhóm có nhắc JWT thay cookie, OpenAPI/Swagger, API versioning và CORS theo từng client. Component Diagram của tôi nên phản ánh các điểm này ở mức giao tiếp component. • Creative Synthesis: Tôi thêm note trên connector client -&gt; IPS Core Service: REST/JSON over HTTPS, Authorization: Bearer JWT, API version /api/v1, OpenAPI contract, CORS allowlist cho Learner Site/Admin Site/Mobile App. Database vẫn nằm sau IPS Core Service, client không truy cập trực tiếp. • Decision Ownership: Quyết định đưa các thay đổi kỹ thuật này vào ghi chú diagram thay vì vẽ thành component quá chi tiết. Lý do: giúp diagram giải thích được cách SOA vận hành mà không làm rối hình. EVIDENCE: Plan tuần 7 SOA-based solution; implementation changes JWT/OpenAPI/CORS/API versioning.</t>
+  </si>
+  <si>
+    <t>DECISION-MAKING | DTC: Abstraction – Document Design Pattern đúng chuẩn GoF trong báo cáo</t>
+  </si>
+  <si>
+    <t>"Làm sao kiểm tra Component Diagram SOA tuần 7 có nhất quán với Package Diagram tuần 5 và code mapping tuần 6 của module Forum + Dictionary? Tôi muốn trace được từ Forum UI đến IPS Core Service rồi tới repository/database."</t>
+  </si>
+  <si>
+    <t>AI RESPONSE (Summary): AI cho rằng Week 7 là kiến trúc thay thế nên không cần nhất quán với package diagram/code hiện tại, có thể vẽ lại tự do. HUMAN DELTA &amp; REFLECTION: • Critical Thinking [Context Misunderstanding]: Alternative Architecture vẫn phải trace được từ hệ thống hiện tại. Nếu SOA diagram không nối được với package/code tuần 5-6, người chấm sẽ khó thấy hướng chuyển đổi khả thi. • Contextualization: Module của tôi đã có Package Diagram (Controllers, Services, Repositories, Data) và code mapping Create Post/Report Content. Trong SOA, các tầng này không biến mất; chúng được gom vào bên trong IPS Core Service. • Creative Synthesis: Tôi kiểm tra traceability: Forum UI/React pages -&gt; REST API endpoint trong IPS Core Service -&gt; PostController/ForumService/PostRepository -&gt; Database Post/Report; Dictionary UI -&gt; DictionaryController/DictionaryService -&gt; DictionaryEntry/SavedWord. Trên diagram SOA, tôi vẽ client chỉ gọi API public, còn package nội bộ nằm trong IPS Core Service. • Decision Ownership: Quyết định giữ tên endpoint/entity/method nhất quán với Week 5-6 khi vẽ SOA. Lý do: chứng minh kiến trúc thay thế là bước tiến hóa từ thiết kế hiện tại, không phải một hệ thống rời rạc. EVIDENCE: Package Diagram Week 5; code snippet mapping Week 6; Component Diagram SOA Week 7.</t>
   </si>
 </sst>
 </file>
@@ -1319,7 +1374,7 @@
     <col min="4" max="4" width="71.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15">
+    <row r="1" spans="1:4" ht="15" customHeight="1">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -1433,6 +1488,120 @@
     <col min="4" max="4" width="69.75" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:4" ht="15" customHeight="1">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="372.6" customHeight="1">
+      <c r="A2" s="6">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="372.6" customHeight="1">
+      <c r="A3" s="6">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="317.45" customHeight="1">
+      <c r="A4" s="6">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="400.15" customHeight="1">
+      <c r="A5" s="6">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="345" customHeight="1">
+      <c r="A6" s="6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="331.15" customHeight="1">
+      <c r="A7" s="6">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>107</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="4.25" customWidth="1"/>
+    <col min="2" max="2" width="24.25" customWidth="1"/>
+    <col min="3" max="3" width="25.375" customWidth="1"/>
+    <col min="4" max="4" width="82" customWidth="1"/>
+  </cols>
+  <sheetData>
     <row r="1" spans="1:4" ht="15">
       <c r="A1" s="5" t="s">
         <v>0</v>
@@ -1447,46 +1616,46 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="372.6" customHeight="1">
+    <row r="2" spans="1:4" ht="345" customHeight="1">
       <c r="A2" s="6">
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>90</v>
+        <v>108</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>91</v>
+        <v>109</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="372.6" customHeight="1">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="358.9" customHeight="1">
       <c r="A3" s="6">
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>93</v>
+        <v>111</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>94</v>
+        <v>112</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="317.45" customHeight="1">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="331.15" customHeight="1">
       <c r="A4" s="6">
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>96</v>
+        <v>114</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>98</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="400.15" customHeight="1">
@@ -1494,41 +1663,41 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>99</v>
+        <v>117</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>100</v>
+        <v>118</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="345" customHeight="1">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="317.45" customHeight="1">
       <c r="A6" s="6">
         <v>5</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>102</v>
+        <v>120</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>103</v>
+        <v>121</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="331.15" customHeight="1">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="345" customHeight="1">
       <c r="A7" s="6">
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>105</v>
+        <v>123</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>106</v>
+        <v>124</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>107</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update audit log week 8
Microservice service discovery
</commit_message>
<xml_diff>
--- a/AI Audit Log_PhamTanHai.xlsx
+++ b/AI Audit Log_PhamTanHai.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="19395" windowHeight="11475" activeTab="7"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="19395" windowHeight="11475" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
@@ -20,13 +20,14 @@
     <sheet name="Week5" sheetId="6" r:id="rId6"/>
     <sheet name="Week6" sheetId="7" r:id="rId7"/>
     <sheet name="Week7" sheetId="8" r:id="rId8"/>
+    <sheet name="Week8" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="144">
   <si>
     <t>STT</t>
   </si>
@@ -449,6 +450,60 @@
   </si>
   <si>
     <t>AI RESPONSE (Summary): AI cho rằng Week 7 là kiến trúc thay thế nên không cần nhất quán với package diagram/code hiện tại, có thể vẽ lại tự do. HUMAN DELTA &amp; REFLECTION: • Critical Thinking [Context Misunderstanding]: Alternative Architecture vẫn phải trace được từ hệ thống hiện tại. Nếu SOA diagram không nối được với package/code tuần 5-6, người chấm sẽ khó thấy hướng chuyển đổi khả thi. • Contextualization: Module của tôi đã có Package Diagram (Controllers, Services, Repositories, Data) và code mapping Create Post/Report Content. Trong SOA, các tầng này không biến mất; chúng được gom vào bên trong IPS Core Service. • Creative Synthesis: Tôi kiểm tra traceability: Forum UI/React pages -&gt; REST API endpoint trong IPS Core Service -&gt; PostController/ForumService/PostRepository -&gt; Database Post/Report; Dictionary UI -&gt; DictionaryController/DictionaryService -&gt; DictionaryEntry/SavedWord. Trên diagram SOA, tôi vẽ client chỉ gọi API public, còn package nội bộ nằm trong IPS Core Service. • Decision Ownership: Quyết định giữ tên endpoint/entity/method nhất quán với Week 5-6 khi vẽ SOA. Lý do: chứng minh kiến trúc thay thế là bước tiến hóa từ thiết kế hiện tại, không phải một hệ thống rời rạc. EVIDENCE: Package Diagram Week 5; code snippet mapping Week 6; Component Diagram SOA Week 7.</t>
+  </si>
+  <si>
+    <t>DECISION-MAKING | DTC: Abstraction – Xác định component chính trong kiến trúc Microservice</t>
+  </si>
+  <si>
+    <t>"Theo kế hoạch tuần 8, tôi phụ trách Component Diagram cho kiến trúc Microservice của IELTSPhobic. Hãy giúp tôi xác định các component chính gồm API Gateway, ServiceRegister, ForumService, VocabService, UserService và các database/service phụ liên quan đến Forum + Dictionary + Vocabulary."</t>
+  </si>
+  <si>
+    <t>AI RESPONSE (Summary): AI đề xuất vẽ một WebAPI lớn, một database chung và thêm ServiceRegister ở cạnh bên cho có đủ thành phần microservice. HUMAN DELTA &amp; REFLECTION: • Critical Thinking [Context Misunderstanding]: Cách này vẫn giống monolith/SOA, chưa phải microservice. Nếu chỉ có một WebAPI lớn thì ServiceRegister gần như vô nghĩa vì không có nhiều service để discover. • Contextualization: Kế hoạch tuần 8 yêu cầu Microservice + Service Discovery, nên diagram phải thể hiện API Gateway, ServiceRegister và nhiều service độc lập. Phần của tôi tập trung vào Forum + Dictionary + Vocabulary, không cần ôm toàn bộ hệ thống quá sâu. • Creative Synthesis: Tôi xác định component chính: Client, API Gateway, ServiceRegister, ForumService, VocabService, UserService, ForumDB/VocabDB hoặc database schema tách theo service, và optional Message Broker nếu cần async. ForumService xử lý Post/Comment/Report; VocabService xử lý DictionaryEntry, VocabularyBook, SavedWord; UserService cung cấp identity/user profile qua API nội bộ. • Decision Ownership: Quyết định vẽ nhiều service độc lập thay vì một WebAPI chung. Lý do: đúng tinh thần microservice và làm rõ vai trò discover service của ServiceRegister. EVIDENCE: Plan tuần 8 yêu cầu Component Diagram Microservice + ServiceRegister.</t>
+  </si>
+  <si>
+    <t>VERIFICATION | DTC: Pattern Recognition – Phân biệt SOA và Microservice + Service Discovery</t>
+  </si>
+  <si>
+    <t>"Ở tuần 7 tôi đã vẽ SOA với IPS Core Service. Sang tuần 8 chuyển sang Microservice + Service Discovery, tôi nên phân biệt hai kiến trúc này thế nào để không vẽ trùng? ServiceRegister xuất hiện ở đâu và có vai trò gì?"</t>
+  </si>
+  <si>
+    <t>AI RESPONSE (Summary): AI nói SOA và Microservice gần như giống nhau, chỉ khác tên gọi, nên có thể dùng lại diagram Week 7 và đổi IPS Core Service thành API Gateway. HUMAN DELTA &amp; REFLECTION: • Critical Thinking [Oversimplification]: Đây là sai khác quan trọng. Week 7 SOA có IPS Core Service lớn dùng chung; Week 8 Microservice phải có nhiều service nhỏ, deploy độc lập, giao tiếp qua Gateway và cần Service Discovery. Nếu chỉ đổi tên, diagram sẽ không thể hiện được mục tiêu scalability. • Contextualization: Kế hoạch dự án ghi rõ Week 8 là Microservice + Service Discovery, phục vụ NF-06 Scalability khi mở rộng nhiều user. Vì vậy ServiceRegister không phải trang trí mà là trung tâm giúp Gateway tìm địa chỉ service runtime. • Creative Synthesis: Tôi phân biệt rõ: SOA Week 7 = nhiều client gọi một IPS Core Service; Microservice Week 8 = client gọi API Gateway, Gateway query ServiceRegister để tìm ForumService/VocabService/UserService, rồi route request đến service phù hợp. • Decision Ownership: Quyết định không reuse nguyên diagram SOA. Tôi dùng lại ý tưởng REST request/response nhưng bổ sung service discovery, service boundary và database ownership theo service. Lý do: thể hiện đúng sự tiến hóa kiến trúc từ SOA sang Microservice. EVIDENCE: Week 7 SOA diagram; Week 8 Microservice plan.</t>
+  </si>
+  <si>
+    <t>PROBLEM-SOLVING | DTC: Algorithms – Đánh số message 1-16 cho luồng discover service</t>
+  </si>
+  <si>
+    <t>"Hãy đề xuất luồng message 1-16 cho Component Diagram Microservice: client gọi API Gateway, Gateway discover ForumService/VocabService qua ServiceRegister, service xử lý request Create Post, Dictionary Lookup, Save Word và trả response."</t>
+  </si>
+  <si>
+    <t>AI RESPONSE (Summary): AI đưa luồng 4 message rất ngắn: Client -&gt; Gateway, Gateway -&gt; Service, Service -&gt; Database, Service -&gt; Client. HUMAN DELTA &amp; REFLECTION: • Critical Thinking: Luồng này mô tả được ý chính nhưng không đáp ứng yêu cầu 'đánh số message 1-16'. Nó cũng bỏ qua bước discover service qua ServiceRegister, là trọng tâm của tuần 8. • Contextualization: Phần của tôi cần thể hiện luồng discover cho Forum + Dictionary/Vocabulary, nên message phải bao gồm Gateway hỏi registry, registry trả instance, Gateway forward request, service xử lý database và response quay lại. • Creative Synthesis: Tôi thiết kế message 1-16 như sau: 1 Client -&gt; API Gateway: POST /forum/posts; 2 Gateway -&gt; ServiceRegister: discover ForumService; 3 ServiceRegister -&gt; Gateway: ForumService instance; 4 Gateway -&gt; ForumService: forward CreatePost; 5 ForumService -&gt; ForumDB: insert Post; 6 ForumDB -&gt; ForumService: save result; 7 ForumService -&gt; Gateway: post created; 8 Gateway -&gt; Client: 201 Created; 9 Client -&gt; Gateway: GET /dictionary?word=...; 10 Gateway -&gt; ServiceRegister: discover VocabService; 11 ServiceRegister -&gt; Gateway: VocabService instance; 12 Gateway -&gt; VocabService: lookup word; 13 VocabService -&gt; VocabDB: query DictionaryEntry; 14 VocabDB -&gt; VocabService: word detail; 15 VocabService -&gt; Gateway: 200 WordDetail; 16 Gateway -&gt; Client: 200 OK. • Decision Ownership: Quyết định dùng đúng 16 message và đánh số trực tiếp trên connector. Lý do: đáp ứng chính xác yêu cầu phân công và giúp giảng viên đọc được service discovery flow. EVIDENCE: Component Diagram Week 8 message list 1-16.</t>
+  </si>
+  <si>
+    <t>VERIFICATION | DTC: Abstraction – Vai trò API Gateway và ServiceRegister trong Component Diagram</t>
+  </si>
+  <si>
+    <t>"Trong Component Diagram Microservice, API Gateway có phải tự xử lý toàn bộ business logic không? Hay Gateway chỉ route request sau khi tìm service qua ServiceRegister? Hãy giải thích để tôi gắn đúng trách nhiệm lên diagram."</t>
+  </si>
+  <si>
+    <t>AI RESPONSE (Summary): AI nói API Gateway có thể chứa authentication, authorization, business logic, validation, database access và gọi thẳng database để giảm số hop. HUMAN DELTA &amp; REFLECTION: • Critical Thinking [Logic Error]: Nếu Gateway chứa business logic và truy cập DB trực tiếp, kiến trúc sẽ quay lại kiểu monolith/god component. Gateway trong microservice nên tập trung vào routing, authentication boundary, rate limiting, request aggregation nhẹ; business rule thuộc service domain. • Contextualization: Với Forum + Vocabulary, logic Create Post, Report Content, Save Word phải nằm trong ForumService/VocabService. Gateway chỉ tìm service qua registry và forward request. • Creative Synthesis: Tôi gắn trách nhiệm trên diagram: API Gateway = entry point, JWT validation, route request, discover service; ServiceRegister = registry of live service instances; ForumService/VocabService = business logic + own data; Database chỉ được truy cập bởi service sở hữu nó. • Decision Ownership: Quyết định không vẽ Gateway truy cập database hoặc xử lý nghiệp vụ sâu. Lý do: giữ đúng nguyên tắc microservice ownership và tránh coupling giữa Gateway với data model nội bộ. CORRECTIVE ACTION: Loại bỏ mũi tên Gateway -&gt; Database; thay bằng Gateway -&gt; ForumService/VocabService. EVIDENCE: Microservice component responsibility; Week 5-6 layered logic trong service.</t>
+  </si>
+  <si>
+    <t>PROBLEM-SOLVING | DTC: Pattern Recognition – Tách ForumService và VocabService đúng bounded context</t>
+  </si>
+  <si>
+    <t>"Module của tôi gồm Forum + Dictionary + Vocabulary. Khi tách microservice, nên gom Dictionary và Vocabulary chung một VocabService hay tách thành DictionaryService và VocabularyService riêng? Tiêu chí tách bounded context là gì?"</t>
+  </si>
+  <si>
+    <t>AI RESPONSE (Summary): AI khuyên tách DictionaryService và VocabularyService thành hai microservice riêng ngay từ đầu để càng nhỏ càng đúng microservice. HUMAN DELTA &amp; REFLECTION: • Critical Thinking [Oversimplification]: Microservice không có nghĩa là tách càng nhỏ càng tốt. Nếu tách quá sớm, communication phức tạp hơn, nhiều API nội bộ hơn và khó quản lý transaction giữa dictionary lookup và saved word. • Contextualization: Dictionary và Vocabulary trong phạm vi của tôi liên quan chặt: DictionaryEntry được dùng để Save Word vào VocabularyBook; SavedWord tham chiếu EntryId. Đây là một bounded context khá gần nhau. Forum thì khác domain hơn, nên tách ForumService riêng là hợp lý. • Creative Synthesis: Tôi quyết định tách ForumService riêng và gom Dictionary + Vocabulary thành VocabService trong diagram Week 8. Nếu sau này dictionary data lớn hoặc cần provider riêng, có thể tách DictionaryService sau, nhưng ở mức thiết kế hiện tại VocabService là cân bằng tốt. • Decision Ownership: Quyết định dùng ForumService + VocabService thay vì tách quá nhiều service. Lý do: giảm coupling liên-service, vẫn thể hiện rõ microservice boundary và giữ diagram đọc được. EVIDENCE: Week 5 schema DictionaryEntry/VocabularyBook/SavedWord; Week 8 scalability design.</t>
+  </si>
+  <si>
+    <t>DECISION-MAKING | DTC: Evaluation – Kiểm tra traceability từ Week 5-7 sang Microservice Week 8</t>
+  </si>
+  <si>
+    <t>"Làm sao kiểm tra Week 8 Microservice Component Diagram vẫn trace được với Package Diagram tuần 5, code snippet tuần 6 và SOA diagram tuần 7? Tôi muốn tránh việc vẽ kiến trúc mới nhưng mất liên hệ với module Forum + Dictionary."</t>
+  </si>
+  <si>
+    <t>AI RESPONSE (Summary): AI cho rằng Week 8 là kiến trúc mới nên không cần giữ tên endpoint/entity từ Week 5-7, có thể đổi tự do cho đẹp diagram. HUMAN DELTA &amp; REFLECTION: • Critical Thinking [Context Misunderstanding]: Kiến trúc mới vẫn phải trace được từ tài liệu trước. Nếu Week 5 có Post/Report/DictionaryEntry/SavedWord, Week 6 có CreatePost/ReportContent, Week 7 có REST endpoint, thì Week 8 nên giữ cùng tên domain để chứng minh continuity. • Contextualization: Module xuyên suốt của tôi là Forum + Dictionary + Vocabulary. Microservice chỉ thay cách deploy và giao tiếp, không thay nghiệp vụ cốt lõi. • Creative Synthesis: Tôi kiểm tra traceability: Package Diagram Week 5 Controllers/Services/Repositories -&gt; trong microservice trở thành internal packages của ForumService/VocabService; code Week 6 PostController/CommentService -&gt; endpoint trong ForumService; SOA Week 7 REST /api/forum/posts và /api/dictionary -&gt; Week 8 route qua API Gateway và discover service. • Decision Ownership: Quyết định giữ tên ForumService, VocabService, Post, Report, DictionaryEntry, SavedWord và endpoint gần giống Week 7. Lý do: người chấm thấy đây là evolution từ design hiện tại sang microservice, không phải vẽ một kiến trúc rời rạc. EVIDENCE: Week 5 Package/Schema; Week 6 Code Mapping; Week 7 SOA HTTP flow; Week 8 Microservice Service Discovery.</t>
   </si>
 </sst>
 </file>
@@ -1602,7 +1657,7 @@
     <col min="4" max="4" width="82" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15">
+    <row r="1" spans="1:4" ht="15" customHeight="1">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -1698,6 +1753,120 @@
       </c>
       <c r="D7" s="6" t="s">
         <v>125</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="4.25" customWidth="1"/>
+    <col min="2" max="2" width="24.25" customWidth="1"/>
+    <col min="3" max="3" width="25.375" customWidth="1"/>
+    <col min="4" max="4" width="82" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="15" customHeight="1">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="345" customHeight="1">
+      <c r="A2" s="6">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="358.9" customHeight="1">
+      <c r="A3" s="6">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="331.15" customHeight="1">
+      <c r="A4" s="6">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="400.15" customHeight="1">
+      <c r="A5" s="6">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="317.45" customHeight="1">
+      <c r="A6" s="6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="345" customHeight="1">
+      <c r="A7" s="6">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>